<commit_message>
added budget and franchise data
</commit_message>
<xml_diff>
--- a/Tomatometer_Certified.xlsx
+++ b/Tomatometer_Certified.xlsx
@@ -3103,12 +3103,12 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>179 Reviews</t>
+          <t>65 Reviews</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -19343,7 +19343,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>192 Reviews</t>
+          <t>191 Reviews</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -21956,17 +21956,17 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>249 Reviews</t>
+          <t>33 Reviews</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>Certified Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -22878,21 +22878,9 @@
       <c r="N132" t="b">
         <v>0</v>
       </c>
-      <c r="O132" t="inlineStr">
-        <is>
-          <t>51%</t>
-        </is>
-      </c>
-      <c r="P132" t="inlineStr">
-        <is>
-          <t>51 Reviews</t>
-        </is>
-      </c>
-      <c r="Q132" t="inlineStr">
-        <is>
-          <t>Rotten</t>
-        </is>
-      </c>
+      <c r="O132" t="inlineStr"/>
+      <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -23265,12 +23253,12 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>146 Reviews</t>
+          <t>145 Reviews</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -23571,9 +23559,21 @@
       <c r="N141" t="b">
         <v>0</v>
       </c>
-      <c r="O141" t="inlineStr"/>
-      <c r="P141" t="inlineStr"/>
-      <c r="Q141" t="inlineStr"/>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>57 Reviews</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Rotten</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -23720,7 +23720,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>136 Reviews</t>
+          <t>135 Reviews</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -26181,17 +26181,17 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>197 Reviews</t>
+          <t>272 Reviews</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Rotten</t>
+          <t>Certified Fresh</t>
         </is>
       </c>
     </row>
@@ -28793,7 +28793,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>196 Reviews</t>
+          <t>197 Reviews</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -33909,21 +33909,9 @@
       <c r="N106" t="b">
         <v>0</v>
       </c>
-      <c r="O106" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="P106" t="inlineStr">
-        <is>
-          <t>187 Reviews</t>
-        </is>
-      </c>
-      <c r="Q106" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -36044,17 +36032,17 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>146 Reviews</t>
+          <t>24 Reviews</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>Rotten</t>
+          <t>Fresh</t>
         </is>
       </c>
     </row>
@@ -46381,12 +46369,12 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>70%</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>91 Reviews</t>
+          <t>100 Reviews</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -46853,9 +46841,21 @@
       <c r="N96" t="b">
         <v>0</v>
       </c>
-      <c r="O96" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
-      <c r="Q96" t="inlineStr"/>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>132 Reviews</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Certified Fresh</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -51030,12 +51030,12 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>36%</t>
         </is>
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>47 Reviews</t>
+          <t>94 Reviews</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
@@ -53941,9 +53941,21 @@
       <c r="N188" t="b">
         <v>0</v>
       </c>
-      <c r="O188" t="inlineStr"/>
-      <c r="P188" t="inlineStr"/>
-      <c r="Q188" t="inlineStr"/>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>132 Reviews</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Rotten</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -56165,7 +56177,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>338 Reviews</t>
+          <t>339 Reviews</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -59227,21 +59239,9 @@
       <c r="N55" t="b">
         <v>0</v>
       </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>83%</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>397 Reviews</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>Certified Fresh</t>
-        </is>
-      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -59545,12 +59545,12 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>233 Reviews</t>
+          <t>235 Reviews</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -60254,21 +60254,9 @@
       <c r="N68" t="b">
         <v>0</v>
       </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>85%</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>41 Reviews</t>
-        </is>
-      </c>
-      <c r="Q68" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -61755,21 +61743,9 @@
       <c r="N87" t="b">
         <v>0</v>
       </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>119 Reviews</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>Rotten</t>
-        </is>
-      </c>
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -63021,17 +62997,17 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>182 Reviews</t>
+          <t>145 Reviews</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Rotten</t>
+          <t>Fresh</t>
         </is>
       </c>
     </row>
@@ -64836,9 +64812,21 @@
       <c r="N126" t="b">
         <v>0</v>
       </c>
-      <c r="O126" t="inlineStr"/>
-      <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr"/>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>72 Reviews</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Rotten</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -66832,12 +66820,12 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>119 Reviews</t>
+          <t>121 Reviews</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
@@ -69094,12 +69082,12 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>120 Reviews</t>
+          <t>132 Reviews</t>
         </is>
       </c>
       <c r="Q182" t="inlineStr">

</xml_diff>